<commit_message>
Preparing new jobs and exxamining main run
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios144.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios144.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +429,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>scenario_index</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>node</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
@@ -461,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>30158.86932882105</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>21877.20611997813</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -587,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>13925.60765435657</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -650,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>26292.3472489202</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>6573.08681223005</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -713,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>56823.46614803323</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -776,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11552.72754785998</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">
@@ -839,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>27224.880712434</v>
+        <v>36844.09611630544</v>
       </c>
     </row>
     <row r="21">
@@ -902,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>35366.79297716976</v>
+        <v>30755.76046864681</v>
       </c>
     </row>
     <row r="24">
@@ -965,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>15439.90977880794</v>
+        <v>10739.47105274393</v>
       </c>
     </row>
     <row r="27">
@@ -1028,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>13021.59707436775</v>
+        <v>23255.36026151579</v>
       </c>
     </row>
     <row r="30">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3255.399268591937</v>
+        <v>5813.840065378947</v>
       </c>
     </row>
     <row r="32">
@@ -1091,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>58800.25721318633</v>
+        <v>43048.73460781306</v>
       </c>
     </row>
     <row r="33">
@@ -1154,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>14203.09214446946</v>
+        <v>10753.51342411154</v>
       </c>
     </row>
     <row r="36">
@@ -1217,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>33730.85142783677</v>
+        <v>26814.71703674526</v>
       </c>
     </row>
     <row r="39">
@@ -1280,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>25246.14634697351</v>
+        <v>10650.39816506652</v>
       </c>
     </row>
     <row r="42">
@@ -1343,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>11114.97390725493</v>
+        <v>6031.558128076127</v>
       </c>
     </row>
     <row r="45">
@@ -1406,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>11791.01111325835</v>
+        <v>16626.27482455417</v>
       </c>
     </row>
     <row r="48">
@@ -1448,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2947.752778314587</v>
+        <v>4156.568706138542</v>
       </c>
     </row>
     <row r="50">
@@ -1469,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>39581.08389513069</v>
+        <v>34807.53319498364</v>
       </c>
     </row>
     <row r="51">
@@ -1532,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>17029.7958865711</v>
+        <v>13678.42749723228</v>
       </c>
     </row>
     <row r="54">
@@ -1595,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>26484.67365024385</v>
+        <v>18189.81943359092</v>
       </c>
     </row>
     <row r="57">
@@ -1658,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>24251.59139929767</v>
+        <v>14407.72223998532</v>
       </c>
     </row>
     <row r="60">
@@ -1721,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>17358.58918472208</v>
+        <v>17996.18288345583</v>
       </c>
     </row>
     <row r="63">
@@ -1784,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>26537.61480407591</v>
+        <v>18645.34219708079</v>
       </c>
     </row>
     <row r="66">
@@ -1826,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>6634.403701018979</v>
+        <v>4661.335549270197</v>
       </c>
     </row>
     <row r="68">
@@ -1847,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>38963.81669557986</v>
+        <v>51012.92307031886</v>
       </c>
     </row>
     <row r="69">
@@ -1910,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>17003.73625109875</v>
+        <v>7157.194301699537</v>
       </c>
     </row>
     <row r="72">

</xml_diff>

<commit_message>
Experiment preparation and plot creation
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios144.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios144.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>27704.71379621089</v>
+        <v>24374.91127531172</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>22993.18933169442</v>
+        <v>16809.94972933953</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14480.10283854169</v>
+        <v>6964.1998280195</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29956.44962014933</v>
+        <v>21041.48666559187</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7489.112405037332</v>
+        <v>5260.371666397967</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>44709.94695541648</v>
+        <v>62018.61096329158</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11177.54061008852</v>
+        <v>11073.66676587308</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>38068.27620371435</v>
+        <v>19280.79870884734</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>29996.34097896187</v>
+        <v>26347.97172369112</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10431.40239120233</v>
+        <v>9032.898708968358</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>22464.07929196216</v>
+        <v>28355.88834170199</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5616.01982299054</v>
+        <v>7088.972085425497</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>41799.86390539659</v>
+        <v>33827.69725282562</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10442.87568333659</v>
+        <v>9613.111007553427</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>25708.39296093324</v>
+        <v>26833.43962692701</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>13655.24507760699</v>
+        <v>24269.86686991857</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7215.794205582797</v>
+        <v>8686.69032201719</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>16241.63626878765</v>
+        <v>23864.22122641126</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4060.409067196913</v>
+        <v>5966.055306602815</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>35573.71667537648</v>
+        <v>52878.73739302095</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>13129.87755012481</v>
+        <v>17883.02456475421</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>18342.61580025829</v>
+        <v>31987.96116891823</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>15818.66491615211</v>
+        <v>26750.06170725983</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>18410.0406738813</v>
+        <v>10944.47964840785</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>17928.01277455997</v>
+        <v>20156.04745465319</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>4482.003193639992</v>
+        <v>5039.011863663297</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>48850.1653181706</v>
+        <v>42054.54002568508</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>7880.490738312205</v>
+        <v>11291.15527167808</v>
       </c>
     </row>
     <row r="72">

</xml_diff>